<commit_message>
Revisa situacoes e regras do mapa de achados
</commit_message>
<xml_diff>
--- a/02-Execucao/05-Comentarios_Gestor/02-Avaliacao_Comentarios_Gestor/fontes-auditoria-pos-comentarios/painel-avaliacao-evidencias.xlsx
+++ b/02-Execucao/05-Comentarios_Gestor/02-Avaliacao_Comentarios_Gestor/fontes-auditoria-pos-comentarios/painel-avaliacao-evidencias.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:IC99"/>
+  <dimension ref="A1:IG99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1602,6 +1602,26 @@
           <t>q0103[D]__pratica</t>
         </is>
       </c>
+      <c r="ID1" t="inlineStr">
+        <is>
+          <t>q2801ext[B]</t>
+        </is>
+      </c>
+      <c r="IE1" t="inlineStr">
+        <is>
+          <t>q2801ext[B]__resposta_afirmada</t>
+        </is>
+      </c>
+      <c r="IF1" t="inlineStr">
+        <is>
+          <t>q2801ext[B]__justificativa</t>
+        </is>
+      </c>
+      <c r="IG1" t="inlineStr">
+        <is>
+          <t>q2801ext[B]__pratica</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2526,6 +2546,26 @@
           <t>os processos de trabalho e os artefatos padronizados estão aderentes às normas legais e infralegais que regem as contratações públicas</t>
         </is>
       </c>
+      <c r="ID13" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="IE13" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="IF13" t="inlineStr">
+        <is>
+          <t>A evidência não contém modelos, minutas ou qualquer artefato padronizado destinado ao planejamento de contratações de TI. Não há referência aos documentos essenciais para a instrução processual desta fase.</t>
+        </is>
+      </c>
+      <c r="IG13" t="inlineStr">
+        <is>
+          <t>são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2753,6 +2793,26 @@
           <t>definiu responsabilidades pelos ativos associados à informação</t>
         </is>
       </c>
+      <c r="ID14" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="IE14" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="IF14" t="inlineStr">
+        <is>
+          <t>Os artefatos disponibilizados, como modelos de Termo de Referência e Matriz de Riscos, possuem caráter genérico e não abrangem as particularidades exigidas para o planejamento de soluções de TI. Ausência de artefatos específicos para a especificação de requisitos de tecnologia, como software e hardware. A documentação apresentada não supre a necessidade de modelos voltados para TI.</t>
+        </is>
+      </c>
+      <c r="IG14" t="inlineStr">
+        <is>
+          <t>são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3314,6 +3374,26 @@
           <t>possui em sua estrutura cargos ou funções formalmente atribuídas à área de tecnologia da informação</t>
         </is>
       </c>
+      <c r="ID17" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="IE17" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="IF17" t="inlineStr">
+        <is>
+          <t>Embora a imagem liste documentos preenchidos em uma contratação específica, isso não comprova a disponibilização de uma biblioteca de artefatos padronizados ou modelos para uso organizacional. A evidência falha em demonstrar a existência de templates ou modelos de referência padronizados.</t>
+        </is>
+      </c>
+      <c r="IG17" t="inlineStr">
+        <is>
+          <t>são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5958,6 +6038,26 @@
           <t>as análises de benefícios, de custos e de riscos subsidiam as decisões relacionadas à seleção e à priorização das iniciativas de TI (projetos e ações)</t>
         </is>
       </c>
+      <c r="ID29" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="IE29" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="IF29" t="inlineStr">
+        <is>
+          <t>Não foram apresentados artefatos padronizados referentes à fase de planejamento, como DFD, ETP ou TR. A documentação enviada limitou-se a uma listagem de processos, sem conter modelos ou templates de trabalho. Faz-se necessária a disponibilização de exemplares ou modelos de artefatos adotados.</t>
+        </is>
+      </c>
+      <c r="IG29" t="inlineStr">
+        <is>
+          <t>são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6459,6 +6559,26 @@
           <t>as áreas demandantes de soluções de TI participam do processo de planejamento de tecnologia da informação</t>
         </is>
       </c>
+      <c r="ID32" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="IE32" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="IF32" t="inlineStr">
+        <is>
+          <t>Foram identificados artefatos como DFD, ETP e Termo de Referência, porém em um contexto de padronização administrativa geral. Não foi possível verificar a existência de modelos ou documentos padronizados próprios para a fase de planejamento de TI. A evidência é insuficiente por não apresentar especificidade para o objeto de TI.</t>
+        </is>
+      </c>
+      <c r="IG32" t="inlineStr">
+        <is>
+          <t>são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -6653,6 +6773,26 @@
           <t>o processo de trabalho para a seleção de fornecedores contempla as etapas, as responsabilidades dos atores envolvidos e os artefatos resultantes de cada etapa</t>
         </is>
       </c>
+      <c r="ID34" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="IE34" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="IF34" t="inlineStr">
+        <is>
+          <t>Não foram disponibilizados modelos ou templates institucionais para artefatos de planejamento, tais como DFD, ETP, ou Matriz de Riscos. A evidência enviada restringe-se a e-mails de solicitação de cotação e propostas de fornecedores, que não comprovem a padronização desses documentos pela instituição.</t>
+        </is>
+      </c>
+      <c r="IG34" t="inlineStr">
+        <is>
+          <t>são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7074,6 +7214,26 @@
           <t>relacionou-se, no perfil profissional, além de requerimentos de ordem legal, um conjunto de competências e habilidades que os ocupantes dos cargos de gestão devem possuir</t>
         </is>
       </c>
+      <c r="ID37" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="IE37" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="IF37" t="inlineStr">
+        <is>
+          <t>A Equipe de Auditoria avalia que não há artefatos padronizados para a fase de planejamento. Os documentos anexados referem-se apenas a atos administrativos pontuais de designação e ajustes orçamentários, não apresentando modelos de DFD, ETP, TR ou Matriz de Riscos. A evidência é insuficiente por tratar de assunto distinto da fase de planejamento de contratações. Faltam modelos ou formulários padronizados para as etapas de planejamento de TI.</t>
+        </is>
+      </c>
+      <c r="IG37" t="inlineStr">
+        <is>
+          <t>são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -7401,6 +7561,26 @@
           <t>possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
         </is>
       </c>
+      <c r="ID38" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="IE38" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="IF38" t="inlineStr">
+        <is>
+          <t>A Equipe de Auditoria conclui que o item não está conforme. Não foram disponibilizados modelos ou exemplos de artefatos padronizados, impossibilitando a verificação de sua existência. A evidência fornecida restringe-se a uma listagem de contratos, sem conter os documentos requisitados. Ausência dos artefatos padronizados de planejamento, como DFD, ETP ou TR.</t>
+        </is>
+      </c>
+      <c r="IG38" t="inlineStr">
+        <is>
+          <t>são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -7595,6 +7775,26 @@
           <t>gerencia (inventaria e controla) os dispositivos conectados em sua rede</t>
         </is>
       </c>
+      <c r="ID40" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="IE40" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="IF40" t="inlineStr">
+        <is>
+          <t>A análise crítica aponta que, apesar de o regulamento interno prever a necessidade de utilização de artefatos padronizados como DFD, ETP e TR, o documento não disponibiliza os modelos ou minutas-padrão efetivamente aplicáveis à fase de planejamento de TI. O próprio normativo determina que tais modelos devem ser instituídos por ordens de serviço ou instruções normativas futuras, as quais não constam nos documentos enviados. A evidência é insuficiente pois não apresenta os instrumentos padronizados concretos voltados à realidade do planejamento de TI.</t>
+        </is>
+      </c>
+      <c r="IG40" t="inlineStr">
+        <is>
+          <t>são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -7802,6 +8002,26 @@
           <t>relacionou-se, no perfil profissional, além de requerimentos de ordem legal, um conjunto de competências e habilidades que os ocupantes dos cargos de gestão devem possuir</t>
         </is>
       </c>
+      <c r="ID41" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="IE41" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="IF41" t="inlineStr">
+        <is>
+          <t>A avaliação realizada conclui que a apresentação de uma única instância de ETP não é suficiente para comprovar a disponibilização institucional de artefatos padronizados. Não foram fornecidos modelos, templates ou normativos que indiquem que tais artefatos são padronizados e disponibilizados para uso recorrente na organização. A lacuna principal reside na ausência de evidência da padronização sistêmica dos artefatos de planejamento.</t>
+        </is>
+      </c>
+      <c r="IG41" t="inlineStr">
+        <is>
+          <t>são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -8644,6 +8864,26 @@
           <t>a área de TI possui atribuições formalizadas relacionadas à governança, planejamento ou gestão de tecnologia da informação</t>
         </is>
       </c>
+      <c r="ID47" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="IE47" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="IF47" t="inlineStr">
+        <is>
+          <t>O documento enviado é um glossário de termos e não disponibiliza artefatos padronizados, tais como modelos, templates ou checklists da organização para a fase de planejamento das contratações. Não foram encontrados exemplos de Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR) ou Matriz de Riscos que comprovem a padronização pela organização auditada. A evidência é insuficiente por tratar apenas de definições conceituais genéricas sem vinculação documental com a entidade.</t>
+        </is>
+      </c>
+      <c r="IG47" t="inlineStr">
+        <is>
+          <t>são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -9158,6 +9398,26 @@
           <t>o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
+      <c r="ID49" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="IE49" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="IF49" t="inlineStr">
+        <is>
+          <t>Não foram disponibilizados artefatos padronizados para o planejamento de contratações de TI. Embora a norma crie unidades responsáveis por contratos, não apresenta os modelos ou documentos padronizados exigidos, como DFD, ETP, TR ou Matriz de Riscos. A evidência é insuficiente pois, apesar de citar atribuições de planejamento, não entrega os modelos necessários ao critério. Faltam os templates de documentos de planejamento específicos para a realidade tecnológica.</t>
+        </is>
+      </c>
+      <c r="IG49" t="inlineStr">
+        <is>
+          <t>são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -11190,6 +11450,26 @@
           <t>possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
         </is>
       </c>
+      <c r="ID65" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="IE65" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="IF65" t="inlineStr">
+        <is>
+          <t>A avaliação indica que não são disponibilizados artefatos padronizados para a fase de planejamento. O documento enviado trata apenas de competências de fiscalização, não oferecendo modelos de DFD, ETP, TR ou Matriz de Riscos. A evidência é insuficiente por não conter tais documentos nem indicação de sua existência. A lacuna consiste na ausência de modelos padronizados para o planejamento de contratações de TI.</t>
+        </is>
+      </c>
+      <c r="IG65" t="inlineStr">
+        <is>
+          <t>são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -11317,6 +11597,26 @@
           <t>o processo de gestão de configuração e ativos está formalizado (a organização instituiu norma interna, guia ou instrumento similar com orientações quanto à execução do processo e definição de responsabilidades)</t>
         </is>
       </c>
+      <c r="ID66" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="IE66" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="IF66" t="inlineStr">
+        <is>
+          <t>A avaliação realizada indica que o item não está conforme, uma vez que não foram apresentados artefatos padronizados para o planejamento de contratações de TI. A evidência restringe-se a citar números de processos sem expor modelos, minutas ou exemplos de documentos como DFD, ETP, TR ou matriz de riscos. A falta de templates ou artefatos de planejamento inviabiliza a constatação da disponibilidade de ferramentas padronizadas.</t>
+        </is>
+      </c>
+      <c r="IG66" t="inlineStr">
+        <is>
+          <t>são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -11584,6 +11884,26 @@
           <t>as análises de benefícios, de custos e de riscos subsidiam as decisões relacionadas à seleção e à priorização das iniciativas de TI (projetos e ações)</t>
         </is>
       </c>
+      <c r="ID67" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="IE67" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="IF67" t="inlineStr">
+        <is>
+          <t>Não foram apresentados artefatos padronizados para a fase de planejamento. O documento enviado restringe-se a um macrofluxo, não contendo modelos, templates ou referências a artefatos como DFD, ETP, TR ou matrizes de risco. A ausência desses documentos impede a avaliação da padronização e da prática de planejamento. Falta a disponibilização de qualquer modelo ou instrumento padronizado para esta etapa.</t>
+        </is>
+      </c>
+      <c r="IG67" t="inlineStr">
+        <is>
+          <t>são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -13549,6 +13869,26 @@
           <t>os gestores são selecionados com base em perfil profissional previamente definido e documentado, e compatível com o cargo ou função para o qual tenha sido indicado</t>
         </is>
       </c>
+      <c r="ID82" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="IE82" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="IF82" t="inlineStr">
+        <is>
+          <t>A evidência apresentada, composta pelo Regimento Interno (página 3), estabelece a competência da Coordenadoria de Informática para a elaboração de Termos de Referência, mas não comprova a existência ou disponibilização de artefatos padronizados para a fase de planejamento, como modelos de DFD, ETP, Matriz de Riscos ou documentos análogos. A atribuição regimental de realizar uma atividade não equivale à disponibilização de templates ou modelos padronizados de suporte ao planejamento. Identifica-se a lacuna referente à falta de evidência da disponibilização ou existência de modelos de documentos padronizados para o planejamento dessas contratações.</t>
+        </is>
+      </c>
+      <c r="IG82" t="inlineStr">
+        <is>
+          <t>são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -13950,6 +14290,26 @@
           <t>possui em sua estrutura cargos ou funções formalmente atribuídas à área de segurança da informação</t>
         </is>
       </c>
+      <c r="ID85" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="IE85" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="IF85" t="inlineStr">
+        <is>
+          <t>A avaliação da Equipe de Auditoria indica que a evidência é insuficiente. Embora haja menção a minutas padronizadas em nível estadual, não constam no processo os artefatos específicos de planejamento de TI (DFD, ETP, TR ou Matriz de Riscos) adotados pelo SEPM. A evidência não demonstra a existência ou utilização desses documentos no órgão. Faltam exemplos ou modelos dos artefatos de planejamento de TI aplicados pelo auditado.</t>
+        </is>
+      </c>
+      <c r="IG85" t="inlineStr">
+        <is>
+          <t>são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -14544,6 +14904,26 @@
           <t>o catálogo contém as metas definidas para cada serviço (p. ex.: prazos de entrega, horários de serviço e de suporte, bem como pontos de contato para solicitação do serviço, envio de sugestões, esclarecimento de dúvidas e reporte de incidentes)</t>
         </is>
       </c>
+      <c r="ID87" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="IE87" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="IF87" t="inlineStr">
+        <is>
+          <t>Embora a norma estabeleça diretrizes para a elaboração de especificações e análises de risco (seção 6), não são disponibilizados ou referenciados modelos e artefatos padronizados para a fase de planejamento. A ausência de templates ou formulários específicos limita a efetiva padronização da documentação. A evidência é insuficiente por faltar a demonstração prática dos modelos de artefatos.</t>
+        </is>
+      </c>
+      <c r="IG87" t="inlineStr">
+        <is>
+          <t>são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -15079,6 +15459,26 @@
           <t>são disponibilizados artefatos padronizados para a fase de seleção de fornecedores, como minutas, checklists, modelos de edital, pareceres, critérios de julgamento ou documentos equivalentes</t>
         </is>
       </c>
+      <c r="ID92" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="IE92" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="IF92" t="inlineStr">
+        <is>
+          <t>A evidência não demonstra a disponibilização de artefatos padronizados voltados especificamente para a fase de planejamento de contratações de TI. Embora o Decreto apresente modelos para aquisições em geral, não constam artefatos com requisitos ou especificações técnicas necessárias para TI, como critérios de segurança, interoperabilidade ou licenciamento. A documentação apresentada é genérica e insuficiente para atender às especificidades do planejamento de tecnologia. Faltam modelos de artefatos que considerem as características e exigências peculiares de bens e serviços de TI.</t>
+        </is>
+      </c>
+      <c r="IG92" t="inlineStr">
+        <is>
+          <t>são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -15940,6 +16340,26 @@
           <t>as áreas demandantes de soluções de TI participam do processo de planejamento de tecnologia da informação</t>
         </is>
       </c>
+      <c r="ID95" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="IE95" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="IF95" t="inlineStr">
+        <is>
+          <t>Não foram disponibilizados artefatos padronizados para a fase de planejamento das contratações de TI. O PDTIC não apresenta templates de Documento de Formalização da Demanda (DFD), Estudo Técnico Preliminar (ETP), Termo de Referência (TR) ou Matriz de Riscos. A evidência é insuficiente pela inexistência de modelos de documentos essenciais para a fase de planejamento.</t>
+        </is>
+      </c>
+      <c r="IG95" t="inlineStr">
+        <is>
+          <t>são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -16279,6 +16699,26 @@
       <c r="EC98" t="inlineStr">
         <is>
           <t>há base(s) de conhecimento que registra(m) erros conhecidos e problemas, de modo a tornar eficiente e efetiva a resolução de incidentes</t>
+        </is>
+      </c>
+      <c r="ID98" t="inlineStr">
+        <is>
+          <t>Não conforme</t>
+        </is>
+      </c>
+      <c r="IE98" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="IF98" t="inlineStr">
+        <is>
+          <t>A Equipe de Auditoria avalia que não há comprovação de padronização documental. Não foram apresentados modelos, templates ou artefatos específicos para a fase de planejamento, coerente com a declaração de inexistência de fluxos formais registrada na página 3. A evidência é insuficiente para atestar a disponibilidade de artefatos. A lacuna reside na ausência de modelos padronizados de DFD, ETP, TR ou Matriz de Riscos.</t>
+        </is>
+      </c>
+      <c r="IG98" t="inlineStr">
+        <is>
+          <t>são disponibilizados artefatos padronizados para a fase de planejamento das contratações de TIC</t>
         </is>
       </c>
     </row>

</xml_diff>